<commit_message>
Interposer around Samtec SSW-120-01-S-D; stack-height check; make_rc2 gate tool
Body 8.51 mm -> 11 mm M2.5 spacers, 20 mm key posts (+2.5 mm margin over pin tips). Socket
contact resistance stays a conservative first-article-measured placeholder. RC2 gate: only
KiCad 10 ERC remains; make_rc2.sh refuses until then.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ENatZXrEDA18PaxUrZWrpi
</commit_message>
<xml_diff>
--- a/OSBAMS_Pi_Power_Interposer_RevA_RC1/bom/OSBAMS_Pi_Power_Interposer_RevA_RC1_BOM.xlsx
+++ b/OSBAMS_Pi_Power_Interposer_RevA_RC1/bom/OSBAMS_Pi_Power_Interposer_RevA_RC1_BOM.xlsx
@@ -521,27 +521,27 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2x20 2.54 mm gold STACKING female header (Pi GPIO), &gt;=3 A/contact, long tails so Pi pins stay reachable for the Waveshare leads</t>
+          <t>Samtec SSW-120-01-S-D: 2x20, 2.54 mm, through-hole vertical receptacle, 30 uin gold / tin tails, body 8.51 mm, tail 2.64 mm, 4.7 A (one pin powered per row). Mounted from the UNDERSIDE, soldered from the top.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Samtec</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>SSW-120-01-S-D</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>OSBAMS_PiPwr:PinSocket_2x20_P2.54mm_RPi_TopView (pad pattern by Pi pin number)</t>
+          <t>OSBAMS_PiPwr:SSW-120-01-S-D_RPi_TopView (pad pattern by Pi pin number, 1.0 mm drill - confirm vs Samtec footprint)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>OPEN - exact MPN with published per-contact current/resistance must be chosen from a datasheet</t>
+          <t>Owner-selected; ordering code/dimensions to re-check vs the SSW-120 product page. Do NOT use SSW-120-04-G-D (14.83 mm tail, no stock)</t>
         </is>
       </c>
     </row>
@@ -556,17 +556,17 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>M2.5 key standoffs/posts (outward side) - length set by the 3D check so a 180-degree fitting cannot seat</t>
+          <t>M2.5 female-female hex standoff, 20 mm (key posts, outward side) + M2.5 screws - length from check_stack_height.py</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>generic</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>M2.5 x 20 mm standoff</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>OPEN - 3D check vs Pi 5 drawing + enclosure</t>
+          <t>Length computed: socket face stays 11.5 mm above the Pi PCB when reversed (pin tips ~9 mm)</t>
         </is>
       </c>
     </row>
@@ -591,17 +591,17 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>M2.5 standoff/spacer + screw to the Pi header-end mounting holes; spacer length = seated height of the chosen stacking socket</t>
+          <t>M2.5 female-female hex standoff, 11 mm (= 8.51 mm socket body + ~2.5 mm Pi header plastic) + M2.5 screws, to the Pi header-end mounting holes</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>generic</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>M2.5 x 11 mm standoff</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>OPEN - depends on socket MPN</t>
+          <t>Standard HAT spacer length; confirm on a physical Pi 5</t>
         </is>
       </c>
     </row>

</xml_diff>